<commit_message>
Actualiza README.md y motor_turnos.py para mejorar la claridad de las reglas de turnos y pausas; agrega métricas de control en la planificación. Modifica planificacion_turnos.ipynb para especificar la versión de Python.
</commit_message>
<xml_diff>
--- a/plantillas/PLANTILLA_MES_EJEMPLO.xlsx
+++ b/plantillas/PLANTILLA_MES_EJEMPLO.xlsx
@@ -22,11 +22,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd-mm-yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="166" formatCode="hh:mm"/>
-    <numFmt numFmtId="167" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="hh:mm"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -85,18 +84,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -475,9 +479,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -527,9 +529,7 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-    </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,7 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -591,6 +592,11 @@
           <t>HORAS_CONTRATO</t>
         </is>
       </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>TURNO_FIJO</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -993,12 +999,15 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Elija un valor de la lista." type="list">
       <formula1>"Activo,Inactivo"</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Elija un valor de la lista." type="list">
       <formula1>"IMAGENES,EXAMEN Y PROCEDIMIENTOS"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Elija un valor de la lista." type="list">
+      <formula1>"Sin sábado,Mañana C/sábado,Tarde C/sábado,Mañana S/sábado,Tarde S/sábado,Intermedio S/sábado"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3347,43 +3356,43 @@
           <t>Mañana C/sábado</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="7" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C2" s="7" t="n">
         <v>0.6875</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="7" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="E2" s="7" t="n">
         <v>0.6875</v>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="F2" s="7" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="G2" s="7" t="n">
         <v>0.6875</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="H2" s="7" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="I2" s="7" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="J2" s="7" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="K2" s="4" t="n">
+      <c r="K2" s="7" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="L2" s="4" t="n">
+      <c r="L2" s="7" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="M2" s="4" t="n">
+      <c r="M2" s="7" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="N2" s="5">
+      <c r="N2" s="8">
         <f>IF(COUNT(B2:C2)=2,(C2-B2)*24-1,0)+IF(COUNT(D2:E2)=2,(E2-D2)*24-1,0)+IF(COUNT(F2:G2)=2,(G2-F2)*24-1,0)+IF(COUNT(H2:I2)=2,(I2-H2)*24-1,0)+IF(COUNT(J2:K2)=2,(K2-J2)*24-1,0)+IF(COUNT(L2:M2)=2,(M2-L2)*24-0.5,0)</f>
         <v/>
       </c>
@@ -3394,43 +3403,43 @@
           <t>Tarde C/sábado</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="7" t="n">
         <v>0.4791666666666667</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="7" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="7" t="n">
         <v>0.4791666666666667</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" s="7" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="F3" s="7" t="n">
         <v>0.4791666666666667</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="G3" s="7" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="H3" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="I3" s="7" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="J3" s="4" t="n">
+      <c r="J3" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="K3" s="4" t="n">
+      <c r="K3" s="7" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="L3" s="4" t="n">
+      <c r="L3" s="7" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="M3" s="4" t="n">
+      <c r="M3" s="7" t="n">
         <v>0.5833333333333334</v>
       </c>
-      <c r="N3" s="5">
+      <c r="N3" s="8">
         <f>IF(COUNT(B3:C3)=2,(C3-B3)*24-1,0)+IF(COUNT(D3:E3)=2,(E3-D3)*24-1,0)+IF(COUNT(F3:G3)=2,(G3-F3)*24-1,0)+IF(COUNT(H3:I3)=2,(I3-H3)*24-1,0)+IF(COUNT(J3:K3)=2,(K3-J3)*24-1,0)+IF(COUNT(L3:M3)=2,(M3-L3)*24-0.5,0)</f>
         <v/>
       </c>
@@ -3441,39 +3450,39 @@
           <t>Mañana S/sábado</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="7" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="7" t="n">
         <v>0.7291666666666666</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="7" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="7" t="n">
         <v>0.7291666666666666</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="F4" s="7" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="G4" s="7" t="n">
         <v>0.7291666666666666</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="H4" s="7" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="I4" s="7" t="n">
         <v>0.7291666666666666</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="J4" s="7" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="K4" s="7" t="n">
         <v>0.7083333333333334</v>
       </c>
-      <c r="L4" s="4" t="n"/>
-      <c r="M4" s="4" t="n"/>
-      <c r="N4" s="5">
+      <c r="L4" s="7" t="n"/>
+      <c r="M4" s="7" t="n"/>
+      <c r="N4" s="8">
         <f>IF(COUNT(B4:C4)=2,(C4-B4)*24-1,0)+IF(COUNT(D4:E4)=2,(E4-D4)*24-1,0)+IF(COUNT(F4:G4)=2,(G4-F4)*24-1,0)+IF(COUNT(H4:I4)=2,(I4-H4)*24-1,0)+IF(COUNT(J4:K4)=2,(K4-J4)*24-1,0)+IF(COUNT(L4:M4)=2,(M4-L4)*24-0.5,0)</f>
         <v/>
       </c>
@@ -3484,39 +3493,39 @@
           <t>Tarde S/sábado</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="7" t="n">
         <v>0.4375</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="7" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="7" t="n">
         <v>0.4375</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="7" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F5" s="7" t="n">
         <v>0.4375</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="G5" s="7" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="H5" s="7" t="n">
         <v>0.4375</v>
       </c>
-      <c r="I5" s="4" t="n">
+      <c r="I5" s="7" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="J5" s="7" t="n">
         <v>0.4583333333333333</v>
       </c>
-      <c r="K5" s="4" t="n">
+      <c r="K5" s="7" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="L5" s="4" t="n"/>
-      <c r="M5" s="4" t="n"/>
-      <c r="N5" s="5">
+      <c r="L5" s="7" t="n"/>
+      <c r="M5" s="7" t="n"/>
+      <c r="N5" s="8">
         <f>IF(COUNT(B5:C5)=2,(C5-B5)*24-1,0)+IF(COUNT(D5:E5)=2,(E5-D5)*24-1,0)+IF(COUNT(F5:G5)=2,(G5-F5)*24-1,0)+IF(COUNT(H5:I5)=2,(I5-H5)*24-1,0)+IF(COUNT(J5:K5)=2,(K5-J5)*24-1,0)+IF(COUNT(L5:M5)=2,(M5-L5)*24-0.5,0)</f>
         <v/>
       </c>
@@ -3527,39 +3536,39 @@
           <t>Intermedio S/sábado</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="7" t="n">
         <v>0.375</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="7" t="n">
         <v>0.7916666666666666</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="7" t="n">
         <v>0.375</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="7" t="n">
         <v>0.7916666666666666</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="F6" s="7" t="n">
         <v>0.375</v>
       </c>
-      <c r="G6" s="4" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="L6" s="4" t="n"/>
-      <c r="M6" s="4" t="n"/>
-      <c r="N6" s="5">
+      <c r="G6" s="7" t="n">
+        <v>0.7916666666666666</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>0.3958333333333333</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>0.7708333333333334</v>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>0.3958333333333333</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>0.7291666666666666</v>
+      </c>
+      <c r="L6" s="7" t="n"/>
+      <c r="M6" s="7" t="n"/>
+      <c r="N6" s="8">
         <f>IF(COUNT(B6:C6)=2,(C6-B6)*24-1,0)+IF(COUNT(D6:E6)=2,(E6-D6)*24-1,0)+IF(COUNT(F6:G6)=2,(G6-F6)*24-1,0)+IF(COUNT(H6:I6)=2,(I6-H6)*24-1,0)+IF(COUNT(J6:K6)=2,(K6-J6)*24-1,0)+IF(COUNT(L6:M6)=2,(M6-L6)*24-0.5,0)</f>
         <v/>
       </c>
@@ -3575,7 +3584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -3699,11 +3708,11 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>La pausa se toma entre 2,0 y 3,0 h después de entrar / volver.</t>
+          <t>La pausa se toma entre 1,5 y 3,0 h después de entrar / volver.</t>
         </is>
       </c>
     </row>
@@ -3724,11 +3733,11 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>No se puede tomar la pausa justo antes de salir.</t>
+          <t>Entre el fin de la 2ª pausa y la salida.</t>
         </is>
       </c>
     </row>
@@ -3804,6 +3813,64 @@
       <c r="C16" t="inlineStr">
         <is>
           <t>Asegura la cobertura de apertura (08:00).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Pausa: hora más temprana</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Las pausas se escalonan cada 15 min desde esta hora.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Colación L-V: hora más temprana</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Colación L-V: hora más temprana si sale a las 16:30 o antes</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Colación L-V: hora fija del turno de cierre</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Para quienes salen a la hora de cierre (la salida más tarde de la hoja TURNOS).</t>
         </is>
       </c>
     </row>
@@ -3849,7 +3916,7 @@
           <t>Lunes a Viernes</t>
         </is>
       </c>
-      <c r="B2" s="6" t="n">
+      <c r="B2" s="9" t="n">
         <v>0.3333333333333333</v>
       </c>
       <c r="C2" t="n">
@@ -3862,7 +3929,7 @@
           <t>Lunes a Viernes</t>
         </is>
       </c>
-      <c r="B3" s="6" t="n">
+      <c r="B3" s="9" t="n">
         <v>0.375</v>
       </c>
       <c r="C3" t="n">
@@ -3875,7 +3942,7 @@
           <t>Lunes a Viernes</t>
         </is>
       </c>
-      <c r="B4" s="6" t="n">
+      <c r="B4" s="9" t="n">
         <v>0.8229166666666666</v>
       </c>
       <c r="C4" t="n">
@@ -3888,7 +3955,7 @@
           <t>Sábado</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="9" t="n">
         <v>0.3333333333333333</v>
       </c>
       <c r="C5" t="n">
@@ -3901,7 +3968,7 @@
           <t>Sábado</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="9" t="n">
         <v>0.5729166666666666</v>
       </c>
       <c r="C6" t="n">

</xml_diff>